<commit_message>
Add Test Case -4 in PO Master
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/ui-test-data.xlsx
+++ b/src/test/resources/testdata/ui-test-data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation Project Backup\Reetrak Automation-Final\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Local Reetrak Automation\QA-Reetrak-Automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD51E1E-9BF5-46EF-92AF-B0938B5D5F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B65C6D-4F8F-4CB2-AD45-B4FADAC265D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="849" firstSheet="3" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="849" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReetrakAdmin" sheetId="27" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2567" uniqueCount="956">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2575" uniqueCount="957">
   <si>
     <t>username</t>
   </si>
@@ -2923,6 +2923,9 @@
   </si>
   <si>
     <t>CODE2346-PRD2346</t>
+  </si>
+  <si>
+    <t>POMaster_TC_04</t>
   </si>
 </sst>
 </file>
@@ -8875,7 +8878,41 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I5" s="9"/>
+      <c r="A5" t="s">
+        <v>956</v>
+      </c>
+      <c r="B5" t="s">
+        <v>777</v>
+      </c>
+      <c r="C5" s="8" t="str">
+        <f>D3</f>
+        <v>TestPO1</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>952</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>953</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>954</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>774</v>
+      </c>
+      <c r="H5" s="17">
+        <v>200</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>955</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="K5" s="8" t="str">
+        <f>CONCATENATE(D5," with batch ",E5, " updated successfully")</f>
+        <v>234PO1 with batch 234BA1 updated successfully</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I6" s="9"/>

</xml_diff>

<commit_message>
Removed the Test Case-4 in PO Master
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/ui-test-data.xlsx
+++ b/src/test/resources/testdata/ui-test-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Local Reetrak Automation\QA-Reetrak-Automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B65C6D-4F8F-4CB2-AD45-B4FADAC265D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA038A63-2D33-4E98-B49B-40040D20D593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="849" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2575" uniqueCount="957">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2567" uniqueCount="956">
   <si>
     <t>username</t>
   </si>
@@ -2923,9 +2923,6 @@
   </si>
   <si>
     <t>CODE2346-PRD2346</t>
-  </si>
-  <si>
-    <t>POMaster_TC_04</t>
   </si>
 </sst>
 </file>
@@ -8878,41 +8875,10 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>956</v>
-      </c>
-      <c r="B5" t="s">
-        <v>777</v>
-      </c>
-      <c r="C5" s="8" t="str">
-        <f>D3</f>
-        <v>TestPO1</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>952</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>953</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>954</v>
-      </c>
-      <c r="G5" s="18" t="s">
-        <v>774</v>
-      </c>
-      <c r="H5" s="17">
-        <v>200</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>955</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="K5" s="8" t="str">
-        <f>CONCATENATE(D5," with batch ",E5, " updated successfully")</f>
-        <v>234PO1 with batch 234BA1 updated successfully</v>
-      </c>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="9"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="I6" s="9"/>

</xml_diff>